<commit_message>
feat: implement AI data assistant backend agent core with tool integration and responsive chat interface
</commit_message>
<xml_diff>
--- a/data/Real Estate Listings.xlsx
+++ b/data/Real Estate Listings.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1001"/>
+  <dimension ref="A1:K1006"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,7 +519,7 @@
         <v>1971</v>
       </c>
       <c r="I2" t="n">
-        <v>351000</v>
+        <v>99999999</v>
       </c>
       <c r="J2" t="n">
         <v>360000</v>
@@ -44850,6 +44850,221 @@
       <c r="K1001" t="inlineStr">
         <is>
           <t>Sold</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>LST-6003</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E1002" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1002" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H1002" t="n">
+        <v>2022</v>
+      </c>
+      <c r="I1002" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J1002" t="inlineStr"/>
+      <c r="K1002" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>LST-6005</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E1003" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1003" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H1003" t="n">
+        <v>2022</v>
+      </c>
+      <c r="I1003" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1003" t="inlineStr"/>
+      <c r="K1003" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>LST-6005</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E1004" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1004" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H1004" t="n">
+        <v>2022</v>
+      </c>
+      <c r="I1004" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1004" t="inlineStr"/>
+      <c r="K1004" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>LST-6008</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E1005" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H1005" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I1005" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1005" t="inlineStr"/>
+      <c r="K1005" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>LST-6008</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>House</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="E1006" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H1006" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I1006" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1006" t="inlineStr"/>
+      <c r="K1006" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>